<commit_message>
Added more data to sheet
</commit_message>
<xml_diff>
--- a/Data.xlsx
+++ b/Data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Yeeti\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Yeeti\Documents\GitHub\Dear-Data-100-Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10295FF4-355A-4783-8124-44547C2A7CB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E781A325-F68F-4478-B0B8-017F1B2ADE4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13695" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="56">
   <si>
     <t>Data No.</t>
   </si>
@@ -55,9 +55,6 @@
     <t>How Angry (1-5)</t>
   </si>
   <si>
-    <t>What I Did</t>
-  </si>
-  <si>
     <t>Game Result (W/L)</t>
   </si>
   <si>
@@ -82,16 +79,115 @@
     <t>Died that round. Killed by Vyse</t>
   </si>
   <si>
-    <t>Bookmarked during buy phase, so may be about round 13</t>
-  </si>
-  <si>
-    <t>Died that round. Killed by dada cee n cee</t>
-  </si>
-  <si>
     <t>Died that round. Spike planted, killed by Sova</t>
   </si>
   <si>
     <t>Alive when bookmarked. Spike planted.</t>
+  </si>
+  <si>
+    <t>Loss</t>
+  </si>
+  <si>
+    <t>Died that round.</t>
+  </si>
+  <si>
+    <t>A player killed me in a annoying way</t>
+  </si>
+  <si>
+    <t>Other Player</t>
+  </si>
+  <si>
+    <t>A player unexpetadtly killed me</t>
+  </si>
+  <si>
+    <t>Mine</t>
+  </si>
+  <si>
+    <t>A player popped outta no where b</t>
+  </si>
+  <si>
+    <t>I died to other player</t>
+  </si>
+  <si>
+    <t>My teammate is trying to blame me for not helping him</t>
+  </si>
+  <si>
+    <t>My gun didn’t shoot properly</t>
+  </si>
+  <si>
+    <t>Game</t>
+  </si>
+  <si>
+    <t>I died as soon as I turned around</t>
+  </si>
+  <si>
+    <t>Sage</t>
+  </si>
+  <si>
+    <t>Corrode</t>
+  </si>
+  <si>
+    <t>Winning</t>
+  </si>
+  <si>
+    <t>I got shot and died through my team mate</t>
+  </si>
+  <si>
+    <t>I died in a way which didn’t make sense</t>
+  </si>
+  <si>
+    <t>I got flashed and died</t>
+  </si>
+  <si>
+    <t>Draw</t>
+  </si>
+  <si>
+    <t>My team doesn’t want to rotate off the other site</t>
+  </si>
+  <si>
+    <t>Teammates</t>
+  </si>
+  <si>
+    <t>Lotus</t>
+  </si>
+  <si>
+    <t>Vyse</t>
+  </si>
+  <si>
+    <t>My team mate literally has no headphones</t>
+  </si>
+  <si>
+    <t>My teammate used his ultimate ability, and does nothing</t>
+  </si>
+  <si>
+    <t>My team is just usless</t>
+  </si>
+  <si>
+    <t>Bind</t>
+  </si>
+  <si>
+    <t>I get killed by two people who used the teleporter</t>
+  </si>
+  <si>
+    <t>The enemy player just killed me and another guy at once</t>
+  </si>
+  <si>
+    <t>Abyss</t>
+  </si>
+  <si>
+    <t>Cypher</t>
+  </si>
+  <si>
+    <t>The enemy player is moving while he killed me</t>
+  </si>
+  <si>
+    <t>I lagged</t>
+  </si>
+  <si>
+    <t>Skye</t>
+  </si>
+  <si>
+    <t>My teammates is trying to shit talk me</t>
   </si>
 </sst>
 </file>
@@ -132,11 +228,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -440,8 +539,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N101"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:M101"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="9" customWidth="1"/>
@@ -450,7 +549,7 @@
     <col min="6" max="6" width="10" customWidth="1"/>
     <col min="7" max="7" width="11" customWidth="1"/>
     <col min="8" max="8" width="17" customWidth="1"/>
-    <col min="9" max="9" width="28" customWidth="1"/>
+    <col min="9" max="9" width="46.06640625" customWidth="1"/>
     <col min="10" max="10" width="13" customWidth="1"/>
     <col min="11" max="11" width="15" customWidth="1"/>
     <col min="12" max="12" width="22" customWidth="1"/>
@@ -458,7 +557,7 @@
     <col min="14" max="14" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -498,11 +597,8 @@
       <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -510,10 +606,10 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2" t="s">
         <v>14</v>
-      </c>
-      <c r="D2" t="s">
-        <v>15</v>
       </c>
       <c r="E2">
         <v>3</v>
@@ -525,13 +621,25 @@
         <v>2</v>
       </c>
       <c r="H2" t="s">
-        <v>16</v>
-      </c>
-      <c r="N2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I2" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="J2" t="s">
+        <v>24</v>
+      </c>
+      <c r="K2" s="3">
+        <v>2</v>
+      </c>
+      <c r="L2" t="s">
+        <v>21</v>
+      </c>
+      <c r="M2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -539,10 +647,10 @@
         <v>1</v>
       </c>
       <c r="C3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" t="s">
         <v>14</v>
-      </c>
-      <c r="D3" t="s">
-        <v>15</v>
       </c>
       <c r="E3">
         <v>5</v>
@@ -554,13 +662,25 @@
         <v>3</v>
       </c>
       <c r="H3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I3" t="s">
+        <v>25</v>
+      </c>
+      <c r="J3" t="s">
+        <v>26</v>
+      </c>
+      <c r="K3" s="3">
+        <v>2</v>
+      </c>
+      <c r="L3" t="s">
+        <v>21</v>
+      </c>
+      <c r="M3" t="s">
         <v>16</v>
       </c>
-      <c r="N3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -568,10 +688,10 @@
         <v>1</v>
       </c>
       <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" t="s">
         <v>14</v>
-      </c>
-      <c r="D4" t="s">
-        <v>15</v>
       </c>
       <c r="E4">
         <v>6</v>
@@ -583,13 +703,25 @@
         <v>4</v>
       </c>
       <c r="H4" t="s">
-        <v>16</v>
-      </c>
-      <c r="N4" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+      <c r="I4" t="s">
+        <v>27</v>
+      </c>
+      <c r="J4" t="s">
+        <v>24</v>
+      </c>
+      <c r="K4" s="3">
+        <v>1</v>
+      </c>
+      <c r="L4" t="s">
+        <v>21</v>
+      </c>
+      <c r="M4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -597,10 +729,10 @@
         <v>1</v>
       </c>
       <c r="C5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" t="s">
         <v>14</v>
-      </c>
-      <c r="D5" t="s">
-        <v>15</v>
       </c>
       <c r="E5">
         <v>7</v>
@@ -612,13 +744,25 @@
         <v>5</v>
       </c>
       <c r="H5" t="s">
-        <v>16</v>
-      </c>
-      <c r="N5" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+      <c r="I5" t="s">
+        <v>28</v>
+      </c>
+      <c r="J5" t="s">
+        <v>26</v>
+      </c>
+      <c r="K5" s="3">
+        <v>1</v>
+      </c>
+      <c r="L5" t="s">
+        <v>21</v>
+      </c>
+      <c r="M5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -626,10 +770,10 @@
         <v>1</v>
       </c>
       <c r="C6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" t="s">
         <v>14</v>
-      </c>
-      <c r="D6" t="s">
-        <v>15</v>
       </c>
       <c r="E6">
         <v>11</v>
@@ -641,13 +785,25 @@
         <v>7</v>
       </c>
       <c r="H6" t="s">
-        <v>16</v>
-      </c>
-      <c r="N6" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+      <c r="I6" t="s">
+        <v>29</v>
+      </c>
+      <c r="J6" t="s">
+        <v>24</v>
+      </c>
+      <c r="K6" s="3">
+        <v>4</v>
+      </c>
+      <c r="L6" t="s">
+        <v>21</v>
+      </c>
+      <c r="M6" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -655,13 +811,13 @@
         <v>1</v>
       </c>
       <c r="C7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D7" t="s">
         <v>14</v>
       </c>
-      <c r="D7" t="s">
-        <v>15</v>
-      </c>
       <c r="E7">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F7">
         <v>4</v>
@@ -670,13 +826,22 @@
         <v>9</v>
       </c>
       <c r="H7" t="s">
-        <v>16</v>
-      </c>
-      <c r="N7" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+      <c r="I7" t="s">
+        <v>30</v>
+      </c>
+      <c r="J7" t="s">
+        <v>31</v>
+      </c>
+      <c r="K7" s="3">
+        <v>2</v>
+      </c>
+      <c r="L7" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -684,10 +849,10 @@
         <v>1</v>
       </c>
       <c r="C8" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8" t="s">
         <v>14</v>
-      </c>
-      <c r="D8" t="s">
-        <v>15</v>
       </c>
       <c r="E8">
         <v>16</v>
@@ -699,13 +864,25 @@
         <v>11</v>
       </c>
       <c r="H8" t="s">
-        <v>16</v>
-      </c>
-      <c r="N8" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+      <c r="I8" t="s">
+        <v>28</v>
+      </c>
+      <c r="J8" t="s">
+        <v>24</v>
+      </c>
+      <c r="K8" s="3">
+        <v>2</v>
+      </c>
+      <c r="L8" t="s">
+        <v>21</v>
+      </c>
+      <c r="M8" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -713,10 +890,10 @@
         <v>1</v>
       </c>
       <c r="C9" t="s">
+        <v>13</v>
+      </c>
+      <c r="D9" t="s">
         <v>14</v>
-      </c>
-      <c r="D9" t="s">
-        <v>15</v>
       </c>
       <c r="E9">
         <v>17</v>
@@ -728,468 +905,909 @@
         <v>12</v>
       </c>
       <c r="H9" t="s">
-        <v>16</v>
-      </c>
-      <c r="N9" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+      <c r="I9" t="s">
+        <v>32</v>
+      </c>
+      <c r="J9" t="s">
+        <v>24</v>
+      </c>
+      <c r="K9" s="3">
+        <v>5</v>
+      </c>
+      <c r="L9" t="s">
+        <v>21</v>
+      </c>
+      <c r="M9" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A10" s="2">
         <v>9</v>
       </c>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B10">
+        <v>2</v>
+      </c>
+      <c r="C10" t="s">
+        <v>34</v>
+      </c>
+      <c r="D10" t="s">
+        <v>33</v>
+      </c>
+      <c r="E10">
+        <v>4</v>
+      </c>
+      <c r="F10">
+        <v>2</v>
+      </c>
+      <c r="G10">
+        <v>1</v>
+      </c>
+      <c r="H10" t="s">
+        <v>35</v>
+      </c>
+      <c r="I10" t="s">
+        <v>36</v>
+      </c>
+      <c r="J10" t="s">
+        <v>24</v>
+      </c>
+      <c r="K10" s="3">
+        <v>2</v>
+      </c>
+      <c r="L10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A11" s="2">
         <v>10</v>
       </c>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B11">
+        <v>2</v>
+      </c>
+      <c r="C11" t="s">
+        <v>34</v>
+      </c>
+      <c r="D11" t="s">
+        <v>33</v>
+      </c>
+      <c r="E11">
+        <v>9</v>
+      </c>
+      <c r="F11">
+        <v>3</v>
+      </c>
+      <c r="G11">
+        <v>5</v>
+      </c>
+      <c r="H11" t="s">
+        <v>15</v>
+      </c>
+      <c r="I11" t="s">
+        <v>37</v>
+      </c>
+      <c r="J11" t="s">
+        <v>24</v>
+      </c>
+      <c r="K11" s="3">
+        <v>3</v>
+      </c>
+      <c r="L11" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A12" s="2">
         <v>11</v>
       </c>
-    </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B12">
+        <v>2</v>
+      </c>
+      <c r="C12" t="s">
+        <v>34</v>
+      </c>
+      <c r="D12" t="s">
+        <v>33</v>
+      </c>
+      <c r="E12">
+        <v>18</v>
+      </c>
+      <c r="F12">
+        <v>10</v>
+      </c>
+      <c r="G12">
+        <v>7</v>
+      </c>
+      <c r="H12" t="s">
+        <v>35</v>
+      </c>
+      <c r="I12" t="s">
+        <v>38</v>
+      </c>
+      <c r="J12" t="s">
+        <v>24</v>
+      </c>
+      <c r="K12" s="3">
+        <v>3</v>
+      </c>
+      <c r="L12" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A13" s="2">
         <v>12</v>
       </c>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B13">
+        <v>2</v>
+      </c>
+      <c r="C13" t="s">
+        <v>34</v>
+      </c>
+      <c r="D13" t="s">
+        <v>33</v>
+      </c>
+      <c r="E13">
+        <v>21</v>
+      </c>
+      <c r="F13">
+        <v>10</v>
+      </c>
+      <c r="G13">
+        <v>10</v>
+      </c>
+      <c r="H13" t="s">
+        <v>39</v>
+      </c>
+      <c r="I13" t="s">
+        <v>40</v>
+      </c>
+      <c r="J13" t="s">
+        <v>41</v>
+      </c>
+      <c r="K13" s="3">
+        <v>4</v>
+      </c>
+      <c r="L13" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A14" s="2">
         <v>13</v>
       </c>
-    </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B14">
+        <v>3</v>
+      </c>
+      <c r="C14" t="s">
+        <v>42</v>
+      </c>
+      <c r="D14" t="s">
+        <v>43</v>
+      </c>
+      <c r="E14">
+        <v>8</v>
+      </c>
+      <c r="F14">
+        <v>0</v>
+      </c>
+      <c r="G14">
+        <v>7</v>
+      </c>
+      <c r="H14" t="s">
+        <v>15</v>
+      </c>
+      <c r="I14" t="s">
+        <v>44</v>
+      </c>
+      <c r="J14" t="s">
+        <v>41</v>
+      </c>
+      <c r="K14" s="3">
+        <v>4</v>
+      </c>
+      <c r="L14" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A15" s="2">
         <v>14</v>
       </c>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B15">
+        <v>3</v>
+      </c>
+      <c r="C15" t="s">
+        <v>42</v>
+      </c>
+      <c r="D15" t="s">
+        <v>43</v>
+      </c>
+      <c r="E15">
+        <v>11</v>
+      </c>
+      <c r="F15">
+        <v>1</v>
+      </c>
+      <c r="G15">
+        <v>9</v>
+      </c>
+      <c r="H15" t="s">
+        <v>15</v>
+      </c>
+      <c r="I15" t="s">
+        <v>45</v>
+      </c>
+      <c r="J15" t="s">
+        <v>41</v>
+      </c>
+      <c r="K15" s="3">
+        <v>4</v>
+      </c>
+      <c r="L15" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A16" s="2">
         <v>15</v>
       </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B16">
+        <v>3</v>
+      </c>
+      <c r="C16" t="s">
+        <v>42</v>
+      </c>
+      <c r="D16" t="s">
+        <v>43</v>
+      </c>
+      <c r="E16">
+        <v>12</v>
+      </c>
+      <c r="F16">
+        <v>2</v>
+      </c>
+      <c r="G16">
+        <v>9</v>
+      </c>
+      <c r="H16" t="s">
+        <v>15</v>
+      </c>
+      <c r="I16" t="s">
+        <v>46</v>
+      </c>
+      <c r="J16" t="s">
+        <v>41</v>
+      </c>
+      <c r="K16" s="3">
+        <v>5</v>
+      </c>
+      <c r="L16" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A17" s="2">
         <v>16</v>
       </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B17">
+        <v>4</v>
+      </c>
+      <c r="C17" t="s">
+        <v>47</v>
+      </c>
+      <c r="D17" t="s">
+        <v>14</v>
+      </c>
+      <c r="E17">
+        <v>3</v>
+      </c>
+      <c r="F17">
+        <v>0</v>
+      </c>
+      <c r="G17">
+        <v>2</v>
+      </c>
+      <c r="H17" t="s">
+        <v>15</v>
+      </c>
+      <c r="I17" t="s">
+        <v>48</v>
+      </c>
+      <c r="J17" t="s">
+        <v>24</v>
+      </c>
+      <c r="K17" s="3">
+        <v>2</v>
+      </c>
+      <c r="L17" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A18" s="2">
         <v>17</v>
       </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B18">
+        <v>4</v>
+      </c>
+      <c r="C18" t="s">
+        <v>47</v>
+      </c>
+      <c r="D18" t="s">
+        <v>14</v>
+      </c>
+      <c r="E18">
+        <v>11</v>
+      </c>
+      <c r="F18">
+        <v>3</v>
+      </c>
+      <c r="G18">
+        <v>7</v>
+      </c>
+      <c r="H18" t="s">
+        <v>15</v>
+      </c>
+      <c r="I18" t="s">
+        <v>49</v>
+      </c>
+      <c r="J18" t="s">
+        <v>24</v>
+      </c>
+      <c r="K18" s="3">
+        <v>3</v>
+      </c>
+      <c r="L18" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A19" s="2">
         <v>18</v>
       </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B19">
+        <v>5</v>
+      </c>
+      <c r="C19" t="s">
+        <v>50</v>
+      </c>
+      <c r="D19" t="s">
+        <v>51</v>
+      </c>
+      <c r="E19">
+        <v>4</v>
+      </c>
+      <c r="F19">
+        <v>1</v>
+      </c>
+      <c r="G19">
+        <v>2</v>
+      </c>
+      <c r="H19" t="s">
+        <v>15</v>
+      </c>
+      <c r="I19" t="s">
+        <v>52</v>
+      </c>
+      <c r="J19" t="s">
+        <v>24</v>
+      </c>
+      <c r="K19" s="3">
+        <v>2</v>
+      </c>
+      <c r="L19" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A20" s="2">
         <v>19</v>
       </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B20">
+        <v>5</v>
+      </c>
+      <c r="C20" t="s">
+        <v>50</v>
+      </c>
+      <c r="D20" t="s">
+        <v>51</v>
+      </c>
+      <c r="E20">
+        <v>10</v>
+      </c>
+      <c r="F20">
+        <v>3</v>
+      </c>
+      <c r="G20">
+        <v>6</v>
+      </c>
+      <c r="H20" t="s">
+        <v>15</v>
+      </c>
+      <c r="I20" t="s">
+        <v>53</v>
+      </c>
+      <c r="J20" t="s">
+        <v>31</v>
+      </c>
+      <c r="K20" s="3">
+        <v>1</v>
+      </c>
+      <c r="L20" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A21" s="2">
         <v>20</v>
       </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B21">
+        <v>5</v>
+      </c>
+      <c r="C21" t="s">
+        <v>50</v>
+      </c>
+      <c r="D21" t="s">
+        <v>51</v>
+      </c>
+      <c r="E21">
+        <v>11</v>
+      </c>
+      <c r="F21">
+        <v>3</v>
+      </c>
+      <c r="G21">
+        <v>7</v>
+      </c>
+      <c r="H21" t="s">
+        <v>15</v>
+      </c>
+      <c r="I21" t="s">
+        <v>30</v>
+      </c>
+      <c r="J21" t="s">
+        <v>31</v>
+      </c>
+      <c r="K21" s="3">
+        <v>2</v>
+      </c>
+      <c r="L21" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A22" s="2">
         <v>21</v>
       </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B22">
+        <v>6</v>
+      </c>
+      <c r="C22" t="s">
+        <v>47</v>
+      </c>
+      <c r="D22" t="s">
+        <v>54</v>
+      </c>
+      <c r="E22">
+        <v>16</v>
+      </c>
+      <c r="F22">
+        <v>6</v>
+      </c>
+      <c r="G22">
+        <v>9</v>
+      </c>
+      <c r="H22" t="s">
+        <v>15</v>
+      </c>
+      <c r="I22" t="s">
+        <v>55</v>
+      </c>
+      <c r="J22" t="s">
+        <v>41</v>
+      </c>
+      <c r="K22" s="3">
+        <v>5</v>
+      </c>
+      <c r="L22" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A23" s="2">
         <v>22</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A24" s="2">
         <v>23</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A25" s="2">
         <v>24</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A26" s="2">
         <v>25</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A27" s="2">
         <v>26</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A28" s="2">
         <v>27</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A29" s="2">
         <v>28</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A30" s="2">
         <v>29</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A31" s="2">
         <v>30</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A32" s="2">
         <v>31</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A33" s="2">
         <v>32</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A34" s="2">
         <v>33</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A35" s="2">
         <v>34</v>
       </c>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A36" s="2">
         <v>35</v>
       </c>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A37" s="2">
         <v>36</v>
       </c>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A38" s="2">
         <v>37</v>
       </c>
     </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A39" s="2">
         <v>38</v>
       </c>
     </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A40" s="2">
         <v>39</v>
       </c>
     </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A41" s="2">
         <v>40</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A42" s="2">
         <v>41</v>
       </c>
     </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A43" s="2">
         <v>42</v>
       </c>
     </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A44" s="2">
         <v>43</v>
       </c>
     </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A45" s="2">
         <v>44</v>
       </c>
     </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A46" s="2">
         <v>45</v>
       </c>
     </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A47" s="2">
         <v>46</v>
       </c>
     </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A48" s="2">
         <v>47</v>
       </c>
     </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A49" s="2">
         <v>48</v>
       </c>
     </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A50" s="2">
         <v>49</v>
       </c>
     </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A51" s="2">
         <v>50</v>
       </c>
     </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A52" s="2">
         <v>51</v>
       </c>
     </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A53" s="2">
         <v>52</v>
       </c>
     </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A54" s="2">
         <v>53</v>
       </c>
     </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A55" s="2">
         <v>54</v>
       </c>
     </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A56" s="2">
         <v>55</v>
       </c>
     </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A57" s="2">
         <v>56</v>
       </c>
     </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A58" s="2">
         <v>57</v>
       </c>
     </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A59" s="2">
         <v>58</v>
       </c>
     </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A60" s="2">
         <v>59</v>
       </c>
     </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A61" s="2">
         <v>60</v>
       </c>
     </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A62" s="2">
         <v>61</v>
       </c>
     </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A63" s="2">
         <v>62</v>
       </c>
     </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A64" s="2">
         <v>63</v>
       </c>
     </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A65" s="2">
         <v>64</v>
       </c>
     </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A66" s="2">
         <v>65</v>
       </c>
     </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A67" s="2">
         <v>66</v>
       </c>
     </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A68" s="2">
         <v>67</v>
       </c>
     </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A69" s="2">
         <v>68</v>
       </c>
     </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A70" s="2">
         <v>69</v>
       </c>
     </row>
-    <row r="71" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A71" s="2">
         <v>70</v>
       </c>
     </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A72" s="2">
         <v>71</v>
       </c>
     </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A73" s="2">
         <v>72</v>
       </c>
     </row>
-    <row r="74" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A74" s="2">
         <v>73</v>
       </c>
     </row>
-    <row r="75" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A75" s="2">
         <v>74</v>
       </c>
     </row>
-    <row r="76" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A76" s="2">
         <v>75</v>
       </c>
     </row>
-    <row r="77" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A77" s="2">
         <v>76</v>
       </c>
     </row>
-    <row r="78" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A78" s="2">
         <v>77</v>
       </c>
     </row>
-    <row r="79" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A79" s="2">
         <v>78</v>
       </c>
     </row>
-    <row r="80" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A80" s="2">
         <v>79</v>
       </c>
     </row>
-    <row r="81" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A81" s="2">
         <v>80</v>
       </c>
     </row>
-    <row r="82" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A82" s="2">
         <v>81</v>
       </c>
     </row>
-    <row r="83" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A83" s="2">
         <v>82</v>
       </c>
     </row>
-    <row r="84" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A84" s="2">
         <v>83</v>
       </c>
     </row>
-    <row r="85" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A85" s="2">
         <v>84</v>
       </c>
     </row>
-    <row r="86" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A86" s="2">
         <v>85</v>
       </c>
     </row>
-    <row r="87" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A87" s="2">
         <v>86</v>
       </c>
     </row>
-    <row r="88" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A88" s="2">
         <v>87</v>
       </c>
     </row>
-    <row r="89" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A89" s="2">
         <v>88</v>
       </c>
     </row>
-    <row r="90" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A90" s="2">
         <v>89</v>
       </c>
     </row>
-    <row r="91" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A91" s="2">
         <v>90</v>
       </c>
     </row>
-    <row r="92" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A92" s="2">
         <v>91</v>
       </c>
     </row>
-    <row r="93" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A93" s="2">
         <v>92</v>
       </c>
     </row>
-    <row r="94" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A94" s="2">
         <v>93</v>
       </c>
     </row>
-    <row r="95" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A95" s="2">
         <v>94</v>
       </c>
     </row>
-    <row r="96" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A96" s="2">
         <v>95</v>
       </c>
     </row>
-    <row r="97" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A97" s="2">
         <v>96</v>
       </c>
     </row>
-    <row r="98" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A98" s="2">
         <v>97</v>
       </c>
     </row>
-    <row r="99" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A99" s="2">
         <v>98</v>
       </c>
     </row>
-    <row r="100" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A100" s="2">
         <v>99</v>
       </c>
     </row>
-    <row r="101" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A101" s="2">
         <v>100</v>
       </c>

</xml_diff>